<commit_message>
fix: separate KOGAS and Joongang databases and restore missing Joongang records
</commit_message>
<xml_diff>
--- a/home/data/Kogas_Material_Inventory.xlsx
+++ b/home/data/Kogas_Material_Inventory.xlsx
@@ -21,10 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -54,9 +51,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -24725,7 +24721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DD4"/>
+  <dimension ref="A1:DD1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25266,794 +25262,8 @@
       </c>
       <c r="DD1" t="inlineStr">
         <is>
-          <t>수량</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46242</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>중앙지사</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>480</v>
-      </c>
-      <c r="D2" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" s="1" t="n">
-        <v>46257.92779054398</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>부장 주진철</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>PAUT MX2(OMNI2-103085)</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>201863</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>2061744</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>PAUT</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>(휴일) 10:00~17:00</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>52,500</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>부장 박광복</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>(휴일) 10:00~17:00</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>52,500</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="inlineStr">
-        <is>
-          <t>81도8458 (스타렉스)</t>
-        </is>
-      </c>
-      <c r="BH2" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="BI2" t="inlineStr">
-        <is>
-          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
-        </is>
-      </c>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>한국지역난방공사 중앙지사</t>
-        </is>
-      </c>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
-      <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>Pipe</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>KS B ISO 13588</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr"/>
-      <c r="BY2" t="inlineStr"/>
-      <c r="BZ2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="CA2" t="inlineStr"/>
-      <c r="CB2" t="inlineStr">
-        <is>
-          <t>일반</t>
-        </is>
-      </c>
-      <c r="CC2" t="inlineStr">
-        <is>
-          <t>300A 이상 (1.0)</t>
-        </is>
-      </c>
-      <c r="CD2" t="inlineStr"/>
-      <c r="CE2" t="inlineStr"/>
-      <c r="CF2" t="inlineStr"/>
-      <c r="CG2" t="n">
-        <v>1</v>
-      </c>
-      <c r="CH2" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="CI2" t="n">
-        <v>383612</v>
-      </c>
-      <c r="CJ2" t="n">
-        <v>665926</v>
-      </c>
-      <c r="CK2" t="n">
-        <v>732518</v>
-      </c>
-      <c r="CL2" t="n">
-        <v>279688</v>
-      </c>
-      <c r="CM2" t="inlineStr"/>
-      <c r="CN2" t="inlineStr"/>
-      <c r="CO2" t="inlineStr"/>
-      <c r="CP2" t="inlineStr"/>
-      <c r="CQ2" t="inlineStr"/>
-      <c r="CR2" t="inlineStr"/>
-      <c r="CS2" t="inlineStr"/>
-      <c r="CT2" t="inlineStr"/>
-      <c r="CU2" t="inlineStr"/>
-      <c r="CV2" t="inlineStr"/>
-      <c r="CW2" t="inlineStr">
-        <is>
-          <t>ORI</t>
-        </is>
-      </c>
-      <c r="CX2" t="n">
-        <v>8</v>
-      </c>
-      <c r="CY2" t="n">
-        <v>0</v>
-      </c>
-      <c r="CZ2" t="inlineStr">
-        <is>
-          <t>400A</t>
-        </is>
-      </c>
-      <c r="DA2" t="inlineStr">
-        <is>
-          <t>열배관</t>
-        </is>
-      </c>
-      <c r="DB2" t="inlineStr"/>
-      <c r="DC2" t="inlineStr"/>
-      <c r="DD2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>46256</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>중앙지사</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>480</v>
-      </c>
-      <c r="D3" t="n">
-        <v>4.0024</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" s="1" t="n">
-        <v>46257.93140291666</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>부장 주진철</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>PAUT MX2(OMNI2-103085)</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>4.0024</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>201862</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" t="n">
-        <v>807934</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>PAUT</t>
-        </is>
-      </c>
-      <c r="V3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>(휴일) 09:00~18:00</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>67,500</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>부장 박광복</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>(휴일) 09:00~18:00</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>67,500</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG3" t="inlineStr">
-        <is>
-          <t>91주8839 (스타렉스) || 95가0175 (스타렉스)</t>
-        </is>
-      </c>
-      <c r="BH3" t="inlineStr">
-        <is>
-          <t>60 || 60</t>
-        </is>
-      </c>
-      <c r="BI3" t="inlineStr">
-        <is>
-          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함 || out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
-        </is>
-      </c>
-      <c r="BJ3" t="inlineStr">
-        <is>
-          <t>||</t>
-        </is>
-      </c>
-      <c r="BK3" t="inlineStr"/>
-      <c r="BL3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM3" t="inlineStr"/>
-      <c r="BN3" t="inlineStr">
-        <is>
-          <t>한국지역난방공사 중앙지사</t>
-        </is>
-      </c>
-      <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr"/>
-      <c r="BQ3" t="inlineStr"/>
-      <c r="BR3" t="inlineStr"/>
-      <c r="BS3" t="inlineStr"/>
-      <c r="BT3" t="inlineStr"/>
-      <c r="BU3" t="inlineStr"/>
-      <c r="BV3" t="inlineStr">
-        <is>
-          <t>Pipe</t>
-        </is>
-      </c>
-      <c r="BW3" t="inlineStr"/>
-      <c r="BX3" t="inlineStr"/>
-      <c r="BY3" t="inlineStr"/>
-      <c r="BZ3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="CA3" t="inlineStr"/>
-      <c r="CB3" t="inlineStr">
-        <is>
-          <t>일반</t>
-        </is>
-      </c>
-      <c r="CC3" t="inlineStr">
-        <is>
-          <t>300A 이상 (1.0)</t>
-        </is>
-      </c>
-      <c r="CD3" t="inlineStr"/>
-      <c r="CE3" t="inlineStr"/>
-      <c r="CF3" t="inlineStr"/>
-      <c r="CG3" t="n">
-        <v>1</v>
-      </c>
-      <c r="CH3" t="n">
-        <v>4.0024</v>
-      </c>
-      <c r="CI3" t="n">
-        <v>150326</v>
-      </c>
-      <c r="CJ3" t="n">
-        <v>260956</v>
-      </c>
-      <c r="CK3" t="n">
-        <v>287051</v>
-      </c>
-      <c r="CL3" t="n">
-        <v>109601</v>
-      </c>
-      <c r="CM3" t="inlineStr"/>
-      <c r="CN3" t="inlineStr"/>
-      <c r="CO3" t="inlineStr"/>
-      <c r="CP3" t="inlineStr"/>
-      <c r="CQ3" t="inlineStr"/>
-      <c r="CR3" t="inlineStr"/>
-      <c r="CS3" t="inlineStr"/>
-      <c r="CT3" t="inlineStr"/>
-      <c r="CU3" t="inlineStr"/>
-      <c r="CV3" t="inlineStr"/>
-      <c r="CW3" t="inlineStr">
-        <is>
-          <t>ORI</t>
-        </is>
-      </c>
-      <c r="CX3" t="n">
-        <v>4</v>
-      </c>
-      <c r="CY3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CZ3" t="inlineStr">
-        <is>
-          <t>300A</t>
-        </is>
-      </c>
-      <c r="DA3" t="inlineStr">
-        <is>
-          <t>열배관</t>
-        </is>
-      </c>
-      <c r="DB3" t="inlineStr"/>
-      <c r="DC3" t="inlineStr"/>
-      <c r="DD3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>46241</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>중앙지사</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>480</v>
-      </c>
-      <c r="D4" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" s="1" t="n">
-        <v>46258.37184412037</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>부장 주진철</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>PAUT MX2(OMNI2-103085)</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>201863</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" t="n">
-        <v>2061744</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>PAUT</t>
-        </is>
-      </c>
-      <c r="V4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>(주간) 09:00~21:00</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>부장 박광복</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>(주간) 09:00~21:00</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
-      <c r="AT4" t="inlineStr"/>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
-      <c r="AX4" t="inlineStr"/>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG4" t="inlineStr">
-        <is>
-          <t>81도8458 (스타렉스)</t>
-        </is>
-      </c>
-      <c r="BH4" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="BI4" t="inlineStr">
-        <is>
-          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
-        </is>
-      </c>
-      <c r="BJ4" t="inlineStr"/>
-      <c r="BK4" t="inlineStr"/>
-      <c r="BL4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM4" t="inlineStr"/>
-      <c r="BN4" t="inlineStr">
-        <is>
-          <t>한국지역난방공사 중앙지사</t>
-        </is>
-      </c>
-      <c r="BO4" t="inlineStr"/>
-      <c r="BP4" t="inlineStr"/>
-      <c r="BQ4" t="inlineStr"/>
-      <c r="BR4" t="inlineStr"/>
-      <c r="BS4" t="inlineStr"/>
-      <c r="BT4" t="inlineStr"/>
-      <c r="BU4" t="inlineStr"/>
-      <c r="BV4" t="inlineStr">
-        <is>
-          <t>Pipe</t>
-        </is>
-      </c>
-      <c r="BW4" t="inlineStr">
-        <is>
-          <t>KS B ISO 13588</t>
-        </is>
-      </c>
-      <c r="BX4" t="inlineStr"/>
-      <c r="BY4" t="inlineStr"/>
-      <c r="BZ4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="CA4" t="inlineStr"/>
-      <c r="CB4" t="inlineStr">
-        <is>
-          <t>일반</t>
-        </is>
-      </c>
-      <c r="CC4" t="inlineStr">
-        <is>
-          <t>300A 이상 (1.0)</t>
-        </is>
-      </c>
-      <c r="CD4" t="inlineStr"/>
-      <c r="CE4" t="inlineStr"/>
-      <c r="CF4" t="inlineStr"/>
-      <c r="CG4" t="n">
-        <v>1</v>
-      </c>
-      <c r="CH4" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="CI4" t="n">
-        <v>383612</v>
-      </c>
-      <c r="CJ4" t="n">
-        <v>665926</v>
-      </c>
-      <c r="CK4" t="n">
-        <v>732518</v>
-      </c>
-      <c r="CL4" t="n">
-        <v>279688</v>
-      </c>
-      <c r="CM4" t="inlineStr"/>
-      <c r="CN4" t="inlineStr"/>
-      <c r="CO4" t="inlineStr"/>
-      <c r="CP4" t="inlineStr"/>
-      <c r="CQ4" t="inlineStr"/>
-      <c r="CR4" t="inlineStr"/>
-      <c r="CS4" t="inlineStr"/>
-      <c r="CT4" t="inlineStr"/>
-      <c r="CU4" t="inlineStr"/>
-      <c r="CV4" t="inlineStr"/>
-      <c r="CW4" t="inlineStr">
-        <is>
-          <t>ORI</t>
-        </is>
-      </c>
-      <c r="CX4" t="n">
-        <v>8</v>
-      </c>
-      <c r="CY4" t="n">
-        <v>0</v>
-      </c>
-      <c r="CZ4" t="inlineStr">
-        <is>
-          <t>400A</t>
-        </is>
-      </c>
-      <c r="DA4" t="inlineStr">
-        <is>
-          <t>열배관</t>
-        </is>
-      </c>
-      <c r="DB4" t="inlineStr"/>
-      <c r="DC4" t="inlineStr"/>
-      <c r="DD4" t="n">
-        <v>0</v>
+          <t>Unnamed:107</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>